<commit_message>
Small changes. Next to fix is date_var
</commit_message>
<xml_diff>
--- a/Crystal_Trays_Library.xlsx
+++ b/Crystal_Trays_Library.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Mastercopy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="10xHis-1TEL-sfGFP-Long-SR-" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DARPin_Crystal_Screen_None" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -15593,11 +15593,7 @@
           <t>Date set:</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>06-06-2025</t>
-        </is>
-      </c>
+      <c r="D1" s="2" t="inlineStr"/>
       <c r="G1" s="19" t="inlineStr">
         <is>
           <t>Enter the top-left subwell concentration:</t>
@@ -15605,7 +15601,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="J1" s="20" t="inlineStr">
@@ -15615,7 +15611,7 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">06-06-2025, Index, 10xHis-1TEL-sfGFP-Long-SR-DARPin, 10.0, 20.0, 1.0, 1TEL, </t>
+          <t xml:space="preserve">, Crystal_Screen, DARPin, 1.0, 1.0, 1.0, 1TEL, </t>
         </is>
       </c>
     </row>
@@ -15637,7 +15633,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>1.0</t>
         </is>
       </c>
     </row>
@@ -15649,7 +15645,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Index</t>
+          <t>Crystal_Screen</t>
         </is>
       </c>
       <c r="G3" s="19" t="inlineStr">
@@ -15672,7 +15668,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>10xHis-1TEL-sfGFP-Long-SR-DARPin</t>
+          <t>DARPin</t>
         </is>
       </c>
     </row>

</xml_diff>